<commit_message>
fix: campos vacíos en PrintableGarantia + fechas y observaciones en Excel PV
- odp.controller: expandir include de garantías con cliente, instaladores y campos faltantes
- PrintableGarantia: cadenas de fallback para instalador, cliente, contacto, teléfono, dirección; ODP muestra solo dígitos; tipo_servicio siempre del padre; eliminado bloque observaciones duplicado
- vitelsa.xlsx: reducir texto OBSERVACIONES a 2 puntos, alineación justificada
- pedido_pv.controller: reestructurar fila 40 — fechas enviada/prometida en rojo (dd/MES/yyyy, tamaño 14) en fila 40, observaciones en B41:S55

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend-api/templates/vitelsa.xlsx
+++ b/backend-api/templates/vitelsa.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>ORDEN DE PEDIDO</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>ALTO</t>
+  </si>
+  <si>
+    <t>FECHA ENVIADA:</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>ENTREGA PROMETIDA:</t>
   </si>
   <si>
     <r>
@@ -173,15 +182,10 @@
         <sz val="13"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">             
+      <t xml:space="preserve">
 *  EXPRESAMENTE AUTORIZO A VITELSA S.A.,  PARA QUE OBTENGA LAS INFORMACIONES Y REFERENCIAS RELATIVAS  A MI PERSONA,  MIS NOMBRES,  APELLIDOS Y DOCUMENTO DE IDENTIFICACIÓN,  A MI COMPORTAMIENTO Y CRÉDITO COMERCIAL,  HÁBITOS DE PAGO,  MANEJO DE MI(S) CUENTA(S) CORRIENTE(S) BANCARIA Y EN GENERAL,  CUMPLIMIENTO DE OBLIGACIONES.     ADEMÁS AUTORIZAMOS IRREVOCABLEMENTE PARA QUE EN EL EVENTO QUE INCUMPLAMOS UNA O CUALQUIERA DE LAS OBLIGACIONES CONTRAIDAS O QUE SE LLEGAREN A CONTRAER, NUESTROS NOMBRES, APELLIDOS Y DOCUMENTO DE IDENTIFICACIÓN, SE INCORPOREN A LOS ARCHIVOS DE DEUDORES MOROSOS DE LA ASOCIACIÓN BANCARIA O CUALQUIER OTRA ENTIDAD SIMILAR.  
 EXHONERAMOS DE TODA RESPONSABILIDAD POR LA INCLUSIÓN DE TALES DATOS A VITELA S.A., ASÍ COMO LA ENTIDAD QUE PRODUZCA EL CORRESPONDIENTE ARCHIVO.         
-* PARA LOS PEDIDOS ENVIADOS A PRODUCCIÓN DESPUÉS DE LAS 11:00 M, SE CONSIDERA COMO DIA INICIAL EL SIGUIENTE DIA HÁBIL.        
-* EL PLAZO DE ENTREGA PARA EL SERVIFLASH ES DE 24 HORAS HÁBILES DE LUNES A VIERNES  
-* LA FORMA DE PAGO DEL SERVIFLASH ES 100% ANTICIPADO, CONSIGNAR EN LAS SIGUIENTES CUENTAS A NOMBRE DE VITELSA S.A.
-BOGOTA CUENTA CORRIENTE CONVENIO 8830 N° CUENTA349-283-465
-BANCOLOMBIA CUENTA AHORROS N° 102-025445-95 CONVENIO 18853
-BANCOLOMBIA CUENTA CORRIENTE N° 625-118-251-07 CONVENIO 18771</t>
+* PARA LOS PEDIDOS ENVIADOS A PRODUCCIÓN DESPUÉS DE LAS 11:00 M, SE CONSIDERA COMO DIA INICIAL EL SIGUIENTE DIA HÁBIL.</t>
     </r>
   </si>
 </sst>
@@ -189,7 +193,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -272,6 +276,15 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <family val="2"/>
       <sz val="13"/>
       <name val="Arial"/>
@@ -303,7 +316,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -688,11 +701,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1117,23 +1137,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2607,346 +2618,354 @@
       <c r="S39" s="134"/>
       <c r="T39" s="2"/>
     </row>
-    <row r="40" ht="60" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="40" ht="20" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B40" s="135" t="s">
         <v>46</v>
       </c>
-      <c r="C40" s="136"/>
-      <c r="D40" s="136"/>
-      <c r="E40" s="136"/>
-      <c r="F40" s="136"/>
-      <c r="G40" s="136"/>
+      <c r="C40" s="135"/>
+      <c r="D40" s="135"/>
+      <c r="E40" s="135"/>
+      <c r="F40" s="135"/>
+      <c r="G40" s="136" t="s">
+        <v>47</v>
+      </c>
       <c r="H40" s="136"/>
       <c r="I40" s="136"/>
       <c r="J40" s="136"/>
-      <c r="K40" s="136"/>
-      <c r="L40" s="136"/>
-      <c r="M40" s="136"/>
-      <c r="N40" s="136"/>
-      <c r="O40" s="136"/>
-      <c r="P40" s="136"/>
+      <c r="K40" s="135" t="s">
+        <v>48</v>
+      </c>
+      <c r="L40" s="135"/>
+      <c r="M40" s="135"/>
+      <c r="N40" s="135"/>
+      <c r="O40" s="135"/>
+      <c r="P40" s="136" t="s">
+        <v>47</v>
+      </c>
       <c r="Q40" s="136"/>
       <c r="R40" s="136"/>
-      <c r="S40" s="137"/>
+      <c r="S40" s="136"/>
       <c r="T40" s="2"/>
     </row>
     <row r="41" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B41" s="138"/>
-      <c r="C41" s="139"/>
-      <c r="D41" s="139"/>
-      <c r="E41" s="139"/>
-      <c r="F41" s="139"/>
-      <c r="G41" s="139"/>
-      <c r="H41" s="139"/>
-      <c r="I41" s="139"/>
-      <c r="J41" s="139"/>
-      <c r="K41" s="139"/>
-      <c r="L41" s="139"/>
-      <c r="M41" s="139"/>
-      <c r="N41" s="139"/>
-      <c r="O41" s="139"/>
-      <c r="P41" s="139"/>
-      <c r="Q41" s="139"/>
-      <c r="R41" s="139"/>
-      <c r="S41" s="140"/>
+      <c r="B41" s="137" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41" s="137"/>
+      <c r="D41" s="137"/>
+      <c r="E41" s="137"/>
+      <c r="F41" s="137"/>
+      <c r="G41" s="137"/>
+      <c r="H41" s="137"/>
+      <c r="I41" s="137"/>
+      <c r="J41" s="137"/>
+      <c r="K41" s="137"/>
+      <c r="L41" s="137"/>
+      <c r="M41" s="137"/>
+      <c r="N41" s="137"/>
+      <c r="O41" s="137"/>
+      <c r="P41" s="137"/>
+      <c r="Q41" s="137"/>
+      <c r="R41" s="137"/>
+      <c r="S41" s="137"/>
       <c r="T41" s="2"/>
     </row>
     <row r="42" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B42" s="138"/>
-      <c r="C42" s="139"/>
-      <c r="D42" s="139"/>
-      <c r="E42" s="139"/>
-      <c r="F42" s="139"/>
-      <c r="G42" s="139"/>
-      <c r="H42" s="139"/>
-      <c r="I42" s="139"/>
-      <c r="J42" s="139"/>
-      <c r="K42" s="139"/>
-      <c r="L42" s="139"/>
-      <c r="M42" s="139"/>
-      <c r="N42" s="139"/>
-      <c r="O42" s="139"/>
-      <c r="P42" s="139"/>
-      <c r="Q42" s="139"/>
-      <c r="R42" s="139"/>
-      <c r="S42" s="140"/>
+      <c r="B42" s="137"/>
+      <c r="C42" s="137"/>
+      <c r="D42" s="137"/>
+      <c r="E42" s="137"/>
+      <c r="F42" s="137"/>
+      <c r="G42" s="137"/>
+      <c r="H42" s="137"/>
+      <c r="I42" s="137"/>
+      <c r="J42" s="137"/>
+      <c r="K42" s="137"/>
+      <c r="L42" s="137"/>
+      <c r="M42" s="137"/>
+      <c r="N42" s="137"/>
+      <c r="O42" s="137"/>
+      <c r="P42" s="137"/>
+      <c r="Q42" s="137"/>
+      <c r="R42" s="137"/>
+      <c r="S42" s="137"/>
       <c r="T42" s="2"/>
     </row>
     <row r="43" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B43" s="138"/>
-      <c r="C43" s="139"/>
-      <c r="D43" s="139"/>
-      <c r="E43" s="139"/>
-      <c r="F43" s="139"/>
-      <c r="G43" s="139"/>
-      <c r="H43" s="139"/>
-      <c r="I43" s="139"/>
-      <c r="J43" s="139"/>
-      <c r="K43" s="139"/>
-      <c r="L43" s="139"/>
-      <c r="M43" s="139"/>
-      <c r="N43" s="139"/>
-      <c r="O43" s="139"/>
-      <c r="P43" s="139"/>
-      <c r="Q43" s="139"/>
-      <c r="R43" s="139"/>
-      <c r="S43" s="140"/>
+      <c r="B43" s="137"/>
+      <c r="C43" s="137"/>
+      <c r="D43" s="137"/>
+      <c r="E43" s="137"/>
+      <c r="F43" s="137"/>
+      <c r="G43" s="137"/>
+      <c r="H43" s="137"/>
+      <c r="I43" s="137"/>
+      <c r="J43" s="137"/>
+      <c r="K43" s="137"/>
+      <c r="L43" s="137"/>
+      <c r="M43" s="137"/>
+      <c r="N43" s="137"/>
+      <c r="O43" s="137"/>
+      <c r="P43" s="137"/>
+      <c r="Q43" s="137"/>
+      <c r="R43" s="137"/>
+      <c r="S43" s="137"/>
       <c r="T43" s="2"/>
     </row>
     <row r="44" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B44" s="138"/>
-      <c r="C44" s="139"/>
-      <c r="D44" s="139"/>
-      <c r="E44" s="139"/>
-      <c r="F44" s="139"/>
-      <c r="G44" s="139"/>
-      <c r="H44" s="139"/>
-      <c r="I44" s="139"/>
-      <c r="J44" s="139"/>
-      <c r="K44" s="139"/>
-      <c r="L44" s="139"/>
-      <c r="M44" s="139"/>
-      <c r="N44" s="139"/>
-      <c r="O44" s="139"/>
-      <c r="P44" s="139"/>
-      <c r="Q44" s="139"/>
-      <c r="R44" s="139"/>
-      <c r="S44" s="140"/>
+      <c r="B44" s="137"/>
+      <c r="C44" s="137"/>
+      <c r="D44" s="137"/>
+      <c r="E44" s="137"/>
+      <c r="F44" s="137"/>
+      <c r="G44" s="137"/>
+      <c r="H44" s="137"/>
+      <c r="I44" s="137"/>
+      <c r="J44" s="137"/>
+      <c r="K44" s="137"/>
+      <c r="L44" s="137"/>
+      <c r="M44" s="137"/>
+      <c r="N44" s="137"/>
+      <c r="O44" s="137"/>
+      <c r="P44" s="137"/>
+      <c r="Q44" s="137"/>
+      <c r="R44" s="137"/>
+      <c r="S44" s="137"/>
       <c r="T44" s="2"/>
     </row>
     <row r="45" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B45" s="138"/>
-      <c r="C45" s="139"/>
-      <c r="D45" s="139"/>
-      <c r="E45" s="139"/>
-      <c r="F45" s="139"/>
-      <c r="G45" s="139"/>
-      <c r="H45" s="139"/>
-      <c r="I45" s="139"/>
-      <c r="J45" s="139"/>
-      <c r="K45" s="139"/>
-      <c r="L45" s="139"/>
-      <c r="M45" s="139"/>
-      <c r="N45" s="139"/>
-      <c r="O45" s="139"/>
-      <c r="P45" s="139"/>
-      <c r="Q45" s="139"/>
-      <c r="R45" s="139"/>
-      <c r="S45" s="140"/>
+      <c r="B45" s="137"/>
+      <c r="C45" s="137"/>
+      <c r="D45" s="137"/>
+      <c r="E45" s="137"/>
+      <c r="F45" s="137"/>
+      <c r="G45" s="137"/>
+      <c r="H45" s="137"/>
+      <c r="I45" s="137"/>
+      <c r="J45" s="137"/>
+      <c r="K45" s="137"/>
+      <c r="L45" s="137"/>
+      <c r="M45" s="137"/>
+      <c r="N45" s="137"/>
+      <c r="O45" s="137"/>
+      <c r="P45" s="137"/>
+      <c r="Q45" s="137"/>
+      <c r="R45" s="137"/>
+      <c r="S45" s="137"/>
       <c r="T45" s="2"/>
     </row>
     <row r="46" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B46" s="138"/>
-      <c r="C46" s="139"/>
-      <c r="D46" s="139"/>
-      <c r="E46" s="139"/>
-      <c r="F46" s="139"/>
-      <c r="G46" s="139"/>
-      <c r="H46" s="139"/>
-      <c r="I46" s="139"/>
-      <c r="J46" s="139"/>
-      <c r="K46" s="139"/>
-      <c r="L46" s="139"/>
-      <c r="M46" s="139"/>
-      <c r="N46" s="139"/>
-      <c r="O46" s="139"/>
-      <c r="P46" s="139"/>
-      <c r="Q46" s="139"/>
-      <c r="R46" s="139"/>
-      <c r="S46" s="140"/>
+      <c r="B46" s="137"/>
+      <c r="C46" s="137"/>
+      <c r="D46" s="137"/>
+      <c r="E46" s="137"/>
+      <c r="F46" s="137"/>
+      <c r="G46" s="137"/>
+      <c r="H46" s="137"/>
+      <c r="I46" s="137"/>
+      <c r="J46" s="137"/>
+      <c r="K46" s="137"/>
+      <c r="L46" s="137"/>
+      <c r="M46" s="137"/>
+      <c r="N46" s="137"/>
+      <c r="O46" s="137"/>
+      <c r="P46" s="137"/>
+      <c r="Q46" s="137"/>
+      <c r="R46" s="137"/>
+      <c r="S46" s="137"/>
       <c r="T46" s="2"/>
     </row>
     <row r="47" ht="12.95" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B47" s="138"/>
-      <c r="C47" s="139"/>
-      <c r="D47" s="139"/>
-      <c r="E47" s="139"/>
-      <c r="F47" s="139"/>
-      <c r="G47" s="139"/>
-      <c r="H47" s="139"/>
-      <c r="I47" s="139"/>
-      <c r="J47" s="139"/>
-      <c r="K47" s="139"/>
-      <c r="L47" s="139"/>
-      <c r="M47" s="139"/>
-      <c r="N47" s="139"/>
-      <c r="O47" s="139"/>
-      <c r="P47" s="139"/>
-      <c r="Q47" s="139"/>
-      <c r="R47" s="139"/>
-      <c r="S47" s="140"/>
+      <c r="B47" s="137"/>
+      <c r="C47" s="137"/>
+      <c r="D47" s="137"/>
+      <c r="E47" s="137"/>
+      <c r="F47" s="137"/>
+      <c r="G47" s="137"/>
+      <c r="H47" s="137"/>
+      <c r="I47" s="137"/>
+      <c r="J47" s="137"/>
+      <c r="K47" s="137"/>
+      <c r="L47" s="137"/>
+      <c r="M47" s="137"/>
+      <c r="N47" s="137"/>
+      <c r="O47" s="137"/>
+      <c r="P47" s="137"/>
+      <c r="Q47" s="137"/>
+      <c r="R47" s="137"/>
+      <c r="S47" s="137"/>
       <c r="T47" s="2"/>
     </row>
     <row r="48" ht="15" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B48" s="138"/>
-      <c r="C48" s="139"/>
-      <c r="D48" s="139"/>
-      <c r="E48" s="139"/>
-      <c r="F48" s="139"/>
-      <c r="G48" s="139"/>
-      <c r="H48" s="139"/>
-      <c r="I48" s="139"/>
-      <c r="J48" s="139"/>
-      <c r="K48" s="139"/>
-      <c r="L48" s="139"/>
-      <c r="M48" s="139"/>
-      <c r="N48" s="139"/>
-      <c r="O48" s="139"/>
-      <c r="P48" s="139"/>
-      <c r="Q48" s="139"/>
-      <c r="R48" s="139"/>
-      <c r="S48" s="140"/>
+      <c r="B48" s="137"/>
+      <c r="C48" s="137"/>
+      <c r="D48" s="137"/>
+      <c r="E48" s="137"/>
+      <c r="F48" s="137"/>
+      <c r="G48" s="137"/>
+      <c r="H48" s="137"/>
+      <c r="I48" s="137"/>
+      <c r="J48" s="137"/>
+      <c r="K48" s="137"/>
+      <c r="L48" s="137"/>
+      <c r="M48" s="137"/>
+      <c r="N48" s="137"/>
+      <c r="O48" s="137"/>
+      <c r="P48" s="137"/>
+      <c r="Q48" s="137"/>
+      <c r="R48" s="137"/>
+      <c r="S48" s="137"/>
       <c r="T48" s="2"/>
     </row>
     <row r="49" ht="15" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B49" s="138"/>
-      <c r="C49" s="139"/>
-      <c r="D49" s="139"/>
-      <c r="E49" s="139"/>
-      <c r="F49" s="139"/>
-      <c r="G49" s="139"/>
-      <c r="H49" s="139"/>
-      <c r="I49" s="139"/>
-      <c r="J49" s="139"/>
-      <c r="K49" s="139"/>
-      <c r="L49" s="139"/>
-      <c r="M49" s="139"/>
-      <c r="N49" s="139"/>
-      <c r="O49" s="139"/>
-      <c r="P49" s="139"/>
-      <c r="Q49" s="139"/>
-      <c r="R49" s="139"/>
-      <c r="S49" s="140"/>
+      <c r="B49" s="137"/>
+      <c r="C49" s="137"/>
+      <c r="D49" s="137"/>
+      <c r="E49" s="137"/>
+      <c r="F49" s="137"/>
+      <c r="G49" s="137"/>
+      <c r="H49" s="137"/>
+      <c r="I49" s="137"/>
+      <c r="J49" s="137"/>
+      <c r="K49" s="137"/>
+      <c r="L49" s="137"/>
+      <c r="M49" s="137"/>
+      <c r="N49" s="137"/>
+      <c r="O49" s="137"/>
+      <c r="P49" s="137"/>
+      <c r="Q49" s="137"/>
+      <c r="R49" s="137"/>
+      <c r="S49" s="137"/>
       <c r="T49" s="2"/>
     </row>
     <row r="50" ht="15" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B50" s="138"/>
-      <c r="C50" s="139"/>
-      <c r="D50" s="139"/>
-      <c r="E50" s="139"/>
-      <c r="F50" s="139"/>
-      <c r="G50" s="139"/>
-      <c r="H50" s="139"/>
-      <c r="I50" s="139"/>
-      <c r="J50" s="139"/>
-      <c r="K50" s="139"/>
-      <c r="L50" s="139"/>
-      <c r="M50" s="139"/>
-      <c r="N50" s="139"/>
-      <c r="O50" s="139"/>
-      <c r="P50" s="139"/>
-      <c r="Q50" s="139"/>
-      <c r="R50" s="139"/>
-      <c r="S50" s="140"/>
+      <c r="B50" s="137"/>
+      <c r="C50" s="137"/>
+      <c r="D50" s="137"/>
+      <c r="E50" s="137"/>
+      <c r="F50" s="137"/>
+      <c r="G50" s="137"/>
+      <c r="H50" s="137"/>
+      <c r="I50" s="137"/>
+      <c r="J50" s="137"/>
+      <c r="K50" s="137"/>
+      <c r="L50" s="137"/>
+      <c r="M50" s="137"/>
+      <c r="N50" s="137"/>
+      <c r="O50" s="137"/>
+      <c r="P50" s="137"/>
+      <c r="Q50" s="137"/>
+      <c r="R50" s="137"/>
+      <c r="S50" s="137"/>
       <c r="T50" s="2"/>
     </row>
     <row r="51" ht="15" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B51" s="138"/>
-      <c r="C51" s="139"/>
-      <c r="D51" s="139"/>
-      <c r="E51" s="139"/>
-      <c r="F51" s="139"/>
-      <c r="G51" s="139"/>
-      <c r="H51" s="139"/>
-      <c r="I51" s="139"/>
-      <c r="J51" s="139"/>
-      <c r="K51" s="139"/>
-      <c r="L51" s="139"/>
-      <c r="M51" s="139"/>
-      <c r="N51" s="139"/>
-      <c r="O51" s="139"/>
-      <c r="P51" s="139"/>
-      <c r="Q51" s="139"/>
-      <c r="R51" s="139"/>
-      <c r="S51" s="140"/>
+      <c r="B51" s="137"/>
+      <c r="C51" s="137"/>
+      <c r="D51" s="137"/>
+      <c r="E51" s="137"/>
+      <c r="F51" s="137"/>
+      <c r="G51" s="137"/>
+      <c r="H51" s="137"/>
+      <c r="I51" s="137"/>
+      <c r="J51" s="137"/>
+      <c r="K51" s="137"/>
+      <c r="L51" s="137"/>
+      <c r="M51" s="137"/>
+      <c r="N51" s="137"/>
+      <c r="O51" s="137"/>
+      <c r="P51" s="137"/>
+      <c r="Q51" s="137"/>
+      <c r="R51" s="137"/>
+      <c r="S51" s="137"/>
       <c r="T51" s="2"/>
     </row>
     <row r="52" ht="12.75" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B52" s="138"/>
-      <c r="C52" s="139"/>
-      <c r="D52" s="139"/>
-      <c r="E52" s="139"/>
-      <c r="F52" s="139"/>
-      <c r="G52" s="139"/>
-      <c r="H52" s="139"/>
-      <c r="I52" s="139"/>
-      <c r="J52" s="139"/>
-      <c r="K52" s="139"/>
-      <c r="L52" s="139"/>
-      <c r="M52" s="139"/>
-      <c r="N52" s="139"/>
-      <c r="O52" s="139"/>
-      <c r="P52" s="139"/>
-      <c r="Q52" s="139"/>
-      <c r="R52" s="139"/>
-      <c r="S52" s="140"/>
+      <c r="B52" s="137"/>
+      <c r="C52" s="137"/>
+      <c r="D52" s="137"/>
+      <c r="E52" s="137"/>
+      <c r="F52" s="137"/>
+      <c r="G52" s="137"/>
+      <c r="H52" s="137"/>
+      <c r="I52" s="137"/>
+      <c r="J52" s="137"/>
+      <c r="K52" s="137"/>
+      <c r="L52" s="137"/>
+      <c r="M52" s="137"/>
+      <c r="N52" s="137"/>
+      <c r="O52" s="137"/>
+      <c r="P52" s="137"/>
+      <c r="Q52" s="137"/>
+      <c r="R52" s="137"/>
+      <c r="S52" s="137"/>
       <c r="T52" s="2"/>
     </row>
-    <row r="53" ht="21" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B53" s="138"/>
-      <c r="C53" s="139"/>
-      <c r="D53" s="139"/>
-      <c r="E53" s="139"/>
-      <c r="F53" s="139"/>
-      <c r="G53" s="139"/>
-      <c r="H53" s="139"/>
-      <c r="I53" s="139"/>
-      <c r="J53" s="139"/>
-      <c r="K53" s="139"/>
-      <c r="L53" s="139"/>
-      <c r="M53" s="139"/>
-      <c r="N53" s="139"/>
-      <c r="O53" s="139"/>
-      <c r="P53" s="139"/>
-      <c r="Q53" s="139"/>
-      <c r="R53" s="139"/>
-      <c r="S53" s="140"/>
+    <row r="53" ht="20" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B53" s="137"/>
+      <c r="C53" s="137"/>
+      <c r="D53" s="137"/>
+      <c r="E53" s="137"/>
+      <c r="F53" s="137"/>
+      <c r="G53" s="137"/>
+      <c r="H53" s="137"/>
+      <c r="I53" s="137"/>
+      <c r="J53" s="137"/>
+      <c r="K53" s="137"/>
+      <c r="L53" s="137"/>
+      <c r="M53" s="137"/>
+      <c r="N53" s="137"/>
+      <c r="O53" s="137"/>
+      <c r="P53" s="137"/>
+      <c r="Q53" s="137"/>
+      <c r="R53" s="137"/>
+      <c r="S53" s="137"/>
       <c r="T53" s="2"/>
     </row>
     <row r="54" ht="18" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B54" s="138"/>
-      <c r="C54" s="139"/>
-      <c r="D54" s="139"/>
-      <c r="E54" s="139"/>
-      <c r="F54" s="139"/>
-      <c r="G54" s="139"/>
-      <c r="H54" s="139"/>
-      <c r="I54" s="139"/>
-      <c r="J54" s="139"/>
-      <c r="K54" s="139"/>
-      <c r="L54" s="139"/>
-      <c r="M54" s="139"/>
-      <c r="N54" s="139"/>
-      <c r="O54" s="139"/>
-      <c r="P54" s="139"/>
-      <c r="Q54" s="139"/>
-      <c r="R54" s="139"/>
-      <c r="S54" s="140"/>
+      <c r="B54" s="137"/>
+      <c r="C54" s="137"/>
+      <c r="D54" s="137"/>
+      <c r="E54" s="137"/>
+      <c r="F54" s="137"/>
+      <c r="G54" s="137"/>
+      <c r="H54" s="137"/>
+      <c r="I54" s="137"/>
+      <c r="J54" s="137"/>
+      <c r="K54" s="137"/>
+      <c r="L54" s="137"/>
+      <c r="M54" s="137"/>
+      <c r="N54" s="137"/>
+      <c r="O54" s="137"/>
+      <c r="P54" s="137"/>
+      <c r="Q54" s="137"/>
+      <c r="R54" s="137"/>
+      <c r="S54" s="137"/>
       <c r="T54" s="2"/>
     </row>
     <row r="55" ht="28.5" customHeight="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B55" s="138"/>
-      <c r="C55" s="139"/>
-      <c r="D55" s="139"/>
-      <c r="E55" s="139"/>
-      <c r="F55" s="139"/>
-      <c r="G55" s="139"/>
-      <c r="H55" s="139"/>
-      <c r="I55" s="139"/>
-      <c r="J55" s="139"/>
-      <c r="K55" s="139"/>
-      <c r="L55" s="139"/>
-      <c r="M55" s="139"/>
-      <c r="N55" s="139"/>
-      <c r="O55" s="139"/>
-      <c r="P55" s="139"/>
-      <c r="Q55" s="139"/>
-      <c r="R55" s="139"/>
-      <c r="S55" s="140"/>
+      <c r="B55" s="137"/>
+      <c r="C55" s="137"/>
+      <c r="D55" s="137"/>
+      <c r="E55" s="137"/>
+      <c r="F55" s="137"/>
+      <c r="G55" s="137"/>
+      <c r="H55" s="137"/>
+      <c r="I55" s="137"/>
+      <c r="J55" s="137"/>
+      <c r="K55" s="137"/>
+      <c r="L55" s="137"/>
+      <c r="M55" s="137"/>
+      <c r="N55" s="137"/>
+      <c r="O55" s="137"/>
+      <c r="P55" s="137"/>
+      <c r="Q55" s="137"/>
+      <c r="R55" s="137"/>
+      <c r="S55" s="137"/>
       <c r="T55" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="53">
+  <mergeCells count="57">
     <mergeCell ref="B2:D7"/>
     <mergeCell ref="E2:Q3"/>
     <mergeCell ref="R2:S7"/>
@@ -2999,7 +3018,11 @@
     <mergeCell ref="R37:S37"/>
     <mergeCell ref="R38:S38"/>
     <mergeCell ref="R39:S39"/>
-    <mergeCell ref="B40:S55"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="K40:O40"/>
+    <mergeCell ref="P40:S40"/>
+    <mergeCell ref="B41:S55"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.1968503937007874" bottom="0.1968503937007874" header="0.07874015748031496" footer="0"/>

</xml_diff>